<commit_message>
registres: especes main propre, 3e pompe Robby prelevee, encaissements dates
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -661,142 +661,197 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>DÉCLARATION URSSAF</t>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Prélèvement personnel</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Un article gardé pour soi sort du stock sans recette. Il ne s'inscrit pas au livre des recettes — il n'y a pas d'encaissement — mais il se note en sortie sur le registre des objets mobiliers, avec la mention « usage personnel ». Sans cette ligne, le stock ne tombe jamais juste.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>Ce qu'on déclare</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Le chiffre d'affaires encaissé sur la période. Total en haut à droite du livre des recettes.</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>VENTES EN ESPÈCES</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Taux</t>
+          <t>Plafond</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>12,3 % de cotisations + 0,1 % de CFP = 12,4 %. À vérifier sur autoentrepreneur.urssaf.fr.</t>
+          <t>1 000 € par transaction entre un professionnel et un particulier résidant en France — art. L112-6 du code monétaire et financier. Aucune vente n'en approche.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Provision</t>
+          <t>La preuve</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>À virer sur un compte séparé à chaque encaissement, pas au trimestre.</t>
+          <t>Une note de vente par transaction : date, article, prix, nom de l'acheteur. Un carnet à souches suffit. C'est elle qui adosse la ligne du registre.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Pas de versement libératoire</t>
+          <t>Le dépôt</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>L'impôt suit le barème après abattement de 71 %. Il tombe l'année suivante — à provisionner aussi.</t>
+          <t>Déposer directement sur le compte professionnel. Passer par le compte personnel puis virer casse le lien entre la vente et le relevé.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>CE QUI RESTE À COMPLÉTER</t>
+          <t>DÉCLARATION URSSAF</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Livre des recettes</t>
+          <t>Ce qu'on déclare</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Le client, le mode de règlement et le canal des sept ventes. La date d'encaissement des deux Havaianas.</t>
+          <t>Le chiffre d'affaires encaissé sur la période. Total en haut à droite du livre des recettes.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Lignes jaunes</t>
+          <t>Taux</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Deux achats sans facture : le lot n°84 (2 pompes Robby, 45 €) et la boîte de 30 boosters Pokémon (65 €).</t>
+          <t>12,3 % de cotisations + 0,1 % de CFP = 12,4 %. À vérifier sur autoentrepreneur.urssaf.fr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Provision</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>À virer sur un compte séparé à chaque encaissement, pas au trimestre.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>OÙ VÉRIFIER</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>URSSAF</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Pas de versement libératoire</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>L'impôt suit le barème après abattement de 71 %. Il tombe l'année suivante — à provisionner aussi.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>Obligations du commerçant</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>entreprendre.service-public.fr</t>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>CE QUI RESTE À COMPLÉTER</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>CGV et droit de la consommation</t>
+          <t>Livre des recettes</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+          <t>Le nom de l'acheteur pour chacune des sept ventes. Le reste est complet : espèces, main propre, dates du 09 et du 10/08/2026.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
+          <t>Lignes jaunes</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Deux achats dont la facture est annoncée : le lot n°84 (3 pompes Robby, 45 €) et la boîte de 30 boosters Pokémon (65 €). Reprendre la date et la référence dès réception.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>OÙ VÉRIFIER</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>URSSAF</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Obligations du commerçant</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>entreprendre.service-public.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>
@@ -935,8 +990,16 @@
       <c r="E6" s="13" t="n">
         <v>135</v>
       </c>
-      <c r="F6" s="12" t="inlineStr"/>
-      <c r="G6" s="12" t="inlineStr"/>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-44194 lot n°9</t>
@@ -971,8 +1034,16 @@
       <c r="E7" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="F7" s="12" t="inlineStr"/>
-      <c r="G7" s="12" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-43716 lot n°103</t>
@@ -998,8 +1069,16 @@
       <c r="E8" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="F8" s="12" t="inlineStr"/>
-      <c r="G8" s="12" t="inlineStr"/>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-43716 lot n°431</t>
@@ -1030,8 +1109,16 @@
       <c r="E9" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="F9" s="12" t="inlineStr"/>
-      <c r="G9" s="12" t="inlineStr"/>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-43716 lot n°170</t>
@@ -1065,8 +1152,16 @@
       <c r="E10" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="F10" s="12" t="inlineStr"/>
-      <c r="G10" s="12" t="inlineStr"/>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-6023 lot n°141</t>
@@ -1097,8 +1192,16 @@
       <c r="E11" s="13" t="n">
         <v>40</v>
       </c>
-      <c r="F11" s="12" t="inlineStr"/>
-      <c r="G11" s="12" t="inlineStr"/>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H11" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-43717 lot n°168</t>
@@ -1115,7 +1218,11 @@
         <f>IF(B12="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B12" s="12" t="inlineStr"/>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="C12" s="12" t="inlineStr"/>
       <c r="D12" s="11" t="inlineStr">
         <is>
@@ -1125,8 +1232,16 @@
       <c r="E12" s="13" t="n">
         <v>28</v>
       </c>
-      <c r="F12" s="12" t="inlineStr"/>
-      <c r="G12" s="12" t="inlineStr"/>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Main propre</t>
+        </is>
+      </c>
       <c r="H12" s="11" t="inlineStr">
         <is>
           <t>Achat : FB2026-5844 lot n°120</t>
@@ -1217,6 +1332,11 @@
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="11" t="n"/>
       <c r="H17" s="11" t="n"/>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Les 493 € encaissés relèvent du 3e trimestre 2026 — déclaration avant le 31 octobre.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10">
@@ -1243,6 +1363,11 @@
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="11" t="n"/>
       <c r="H19" s="11" t="n"/>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>VENTES EN ESPÈCES — CE QU'IL FAUT GARDER</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="10">
@@ -1256,6 +1381,11 @@
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
       <c r="H20" s="11" t="n"/>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>Légal sans limite entre un professionnel et un particulier résidant en France jusqu'à 1 000 €</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="10">
@@ -1269,6 +1399,11 @@
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
       <c r="H21" s="11" t="n"/>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>par transaction (art. L112-6 du code monétaire et financier). Toutes les ventes sont loin du seuil.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="10">
@@ -1282,6 +1417,7 @@
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
       <c r="H22" s="11" t="n"/>
+      <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10">
@@ -1295,6 +1431,11 @@
       <c r="F23" s="11" t="n"/>
       <c r="G23" s="11" t="n"/>
       <c r="H23" s="11" t="n"/>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>La preuve d'une vente en espèces, c'est le registre plus le dépôt bancaire. Trois réflexes :</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="10">
@@ -1308,6 +1449,11 @@
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
       <c r="H24" s="11" t="n"/>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. Une note de vente par transaction — date, article, prix, nom de l'acheteur. Un carnet suffit.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="10">
@@ -1321,6 +1467,11 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
       <c r="H25" s="11" t="n"/>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. Déposer sur le compte professionnel, pas sur le compte personnel : le détour brouille la piste.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="10">
@@ -1334,6 +1485,11 @@
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
       <c r="H26" s="11" t="n"/>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. Déposer par montants qui recoupent le registre, pour que le relevé confirme les lignes.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="10">
@@ -6526,7 +6682,7 @@
       </c>
       <c r="D45" s="12" t="inlineStr">
         <is>
-          <t>Lot n°84 — Lot de 2 pompes immergées ROBBY VP550W</t>
+          <t>Lot n°84 — Lot de 3 pompes immergées ROBBY VP550W</t>
         </is>
       </c>
       <c r="E45" s="17" t="n">
@@ -10345,7 +10501,11 @@
           <t>Carte</t>
         </is>
       </c>
-      <c r="I6" s="20" t="inlineStr"/>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
       <c r="J6" s="21" t="n">
         <v>28</v>
       </c>
@@ -11809,12 +11969,12 @@
       </c>
       <c r="D40" s="12" t="inlineStr">
         <is>
-          <t>Facture à retrouver</t>
+          <t>Facture en attente de réception</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Lot de 2 pompes immergées ROBBY VP550W</t>
+          <t>Lot de 3 pompes immergées ROBBY VP550W</t>
         </is>
       </c>
       <c r="F40" s="12" t="inlineStr">
@@ -11832,7 +11992,11 @@
       </c>
       <c r="I40" s="12" t="inlineStr"/>
       <c r="J40" s="17" t="inlineStr"/>
-      <c r="K40" s="12" t="inlineStr"/>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>3 pompes — 1 prélevée pour usage personnel, sans contrepartie ; 2 restent en stock</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="16">
@@ -11847,7 +12011,7 @@
       </c>
       <c r="D41" s="12" t="inlineStr">
         <is>
-          <t>Facture à retrouver</t>
+          <t>Facture en attente de réception</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">

</xml_diff>

<commit_message>
pokemon: libelles explicites sur les quantites
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -6504,7 +6504,7 @@
       </c>
       <c r="D39" s="11" t="inlineStr">
         <is>
-          <t>Booster Box Pokémon MEGA Nihil Zero (Munikis Zero) M3 — 30 boosters</t>
+          <t>1 booster box Pokémon MEGA Nihil Zero (Munikis Zero) M3 — 30 boosters de 5 cartes</t>
         </is>
       </c>
       <c r="E39" s="13" t="n">
@@ -6538,7 +6538,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>Booster Pokémon High Class Pack MEGA Dream ex M2a — 10 cartes</t>
+          <t>1 booster Pokémon High Class Pack MEGA Dream ex M2a — 10 cartes dans le booster</t>
         </is>
       </c>
       <c r="E40" s="13" t="n">
@@ -6572,7 +6572,7 @@
       </c>
       <c r="D41" s="11" t="inlineStr">
         <is>
-          <t>Boosters Pokémon MEGA Storm Emeralda M6 ×2 — 5 cartes chacun</t>
+          <t>2 boosters Pokémon MEGA Storm Emeralda M6 — 5 cartes chacun</t>
         </is>
       </c>
       <c r="E41" s="13" t="n">
@@ -12076,7 +12076,7 @@
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>Booster Box Pokémon MEGA Nihil Zero (Munikis Zero) M3 — 30 boosters</t>
+          <t>1 booster box Pokémon MEGA Nihil Zero (Munikis Zero) M3 — 30 boosters de 5 cartes</t>
         </is>
       </c>
       <c r="F38" s="11" t="inlineStr">
@@ -12118,7 +12118,7 @@
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>Booster Pokémon High Class Pack MEGA Dream ex M2a — 10 cartes</t>
+          <t>1 booster Pokémon High Class Pack MEGA Dream ex M2a — 10 cartes dans le booster</t>
         </is>
       </c>
       <c r="F39" s="11" t="inlineStr">
@@ -12164,7 +12164,7 @@
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>Boosters Pokémon MEGA Storm Emeralda M6 ×2 — 5 cartes chacun</t>
+          <t>2 boosters Pokémon MEGA Storm Emeralda M6 — 5 cartes chacun</t>
         </is>
       </c>
       <c r="F40" s="11" t="inlineStr">

</xml_diff>

<commit_message>
charges: abonnement Claude 22 EUR/mois, seuil de CA mensuel, dates de prelevement
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -1523,7 +1523,7 @@
       <c r="H28" s="11" t="n"/>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>Pompe ROBBY VP550W ligne 131 — gardée</t>
+          <t>Pompe ROBBY VP550W ligne 131 — gardée, 26/07/2026</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       <c r="H29" s="11" t="n"/>
       <c r="J29" s="8" t="inlineStr">
         <is>
-          <t>Booster High Class MEGA Dream ex M2a — gardé</t>
+          <t>Booster High Class MEGA Dream ex M2a — gardé, 03/08/2026</t>
         </is>
       </c>
     </row>
@@ -10759,7 +10759,11 @@
           <t>Carte</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr"/>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
       <c r="J8" s="12" t="inlineStr"/>
       <c r="K8" s="11" t="inlineStr">
         <is>
@@ -12141,7 +12145,11 @@
           <t>Carte</t>
         </is>
       </c>
-      <c r="I39" s="11" t="inlineStr"/>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>03/08/2026</t>
+        </is>
+      </c>
       <c r="J39" s="12" t="inlineStr"/>
       <c r="K39" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
apport personnel de 150,50 EUR couvrant les quatre prelevements
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -671,209 +671,245 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Le remboursement du prélèvement</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Remettre l'argent sur le compte pro n'est pas obligatoire — il n'y a qu'une personne juridique. Mais c'est une bonne pratique : sans ça, le stock fond et la caisse ne suit pas. Verser le COÛT D'ACHAT, pas le prix de vente : l'entreprise récupère ce qu'elle a payé, ni plus ni moins.</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>VENTES EN ESPÈCES</t>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Apport, pas recette</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Le virement du compte personnel vers le compte professionnel est un APPORT. Aucun chiffre d'affaires, aucune URSSAF, rien à déclarer. Le libeller « apport personnel » : sur un relevé pro, une somme qui arrive sans libellé ressemble à un encaissement client introuvable au livre des recettes.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Apport enregistré</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>150,50 € versés en apport personnel, couvrant au coût les quatre prélèvements : Hoka 65,37 € + Nike 52,77 € + pompe Robby ligne 131 19,41 € + booster High Class 12,95 €.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>VENTES EN ESPÈCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>Plafond</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>1 000 € par transaction entre un professionnel et un particulier résidant en France — art. L112-6 du code monétaire et financier. Aucune vente n'en approche.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>La preuve</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Une note de vente par transaction : date, article, prix, nom de l'acheteur. Un carnet à souches suffit. C'est elle qui adosse la ligne du registre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Le dépôt</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Déposer directement sur le compte professionnel. Passer par le compte personnel puis virer casse le lien entre la vente et le relevé.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>DÉCLARATION URSSAF</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Ce qu'on déclare</t>
+          <t>Le dépôt</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Le chiffre d'affaires encaissé sur la période. Total en haut à droite du livre des recettes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Taux</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>12,3 % de cotisations + 0,1 % de CFP = 12,4 %. À vérifier sur autoentrepreneur.urssaf.fr.</t>
+          <t>Déposer directement sur le compte professionnel. Passer par le compte personnel puis virer casse le lien entre la vente et le relevé.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Provision</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>À virer sur un compte séparé à chaque encaissement, pas au trimestre.</t>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>DÉCLARATION URSSAF</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Pas de versement libératoire</t>
+          <t>Ce qu'on déclare</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>L'impôt suit le barème après abattement de 71 %. Il tombe l'année suivante — à provisionner aussi.</t>
+          <t>Le chiffre d'affaires encaissé sur la période. Total en haut à droite du livre des recettes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Taux</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>12,3 % de cotisations + 0,1 % de CFP = 12,4 %. À vérifier sur autoentrepreneur.urssaf.fr.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>CE QUI RESTE À COMPLÉTER</t>
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Provision</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>À virer sur un compte séparé à chaque encaissement, pas au trimestre.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Livre des recettes</t>
+          <t>Pas de versement libératoire</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>Complet, sauf l'acheteur des deux paires de Havaianas. Quatre ventes à Mme Aouimeur Siham le 09/08, espèces, main propre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="3" t="inlineStr">
-        <is>
-          <t>Plus aucune ligne jaune</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
+          <t>L'impôt suit le barème après abattement de 71 %. Il tombe l'année suivante — à provisionner aussi.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Défauts déclarés</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>CE QUI RESTE À COMPLÉTER</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Import du Japon</t>
+          <t>Livre des recettes</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>La facture Meccha Japan #FA429713 ne porte aucune TVA. Si La Poste a réclamé la TVA à 20 % et des frais de dossier à la livraison, ce montant s'ajoute au coût d'achat : le noter en ligne séparée.</t>
+          <t>Complet, sauf l'acheteur des deux paires de Havaianas. Quatre ventes à Mme Aouimeur Siham le 09/08, espèces, main propre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Plus aucune ligne jaune</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>OÙ VÉRIFIER</t>
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Défauts déclarés</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>URSSAF</t>
+          <t>Import du Japon</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>Obligations du commerçant</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>entreprendre.service-public.fr</t>
+          <t>La facture Meccha Japan #FA429713 ne porte aucune TVA. Si La Poste a réclamé la TVA à 20 % et des frais de dossier à la livraison, ce montant s'ajoute au coût d'achat : le noter en ligne séparée.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>CGV et droit de la consommation</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>OÙ VÉRIFIER</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
+          <t>URSSAF</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Obligations du commerçant</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>entreprendre.service-public.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>

</xml_diff>

<commit_message>
Havaianas: ventes Vinted consignees, les 10 restantes passent a 18 EUR
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Objets mobiliers" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$H$310</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Livre des recettes'!$A$5:$H$311</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Registre des achats'!$A$5:$G$350</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Objets mobiliers'!$A$5:$K$345</definedName>
   </definedNames>
@@ -77,7 +77,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -87,11 +87,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001A1A1A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF4CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -126,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -145,12 +140,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -820,96 +814,108 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Complet, sauf l'acheteur des deux paires de Havaianas. Quatre ventes à Mme Aouimeur Siham le 09/08, espèces, main propre.</t>
+          <t>Complet. Quatre ventes à Mme Aouimeur Siham le 09/08 en espèces et main propre, deux paires de Havaianas sur Vinted encaissées le 10/08.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Plus aucune ligne jaune</t>
+          <t>Ventes Vinted</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
+          <t>Sur un compte particulier, le vendeur ne paie pas de commission et l'acheteur paie le port : le prix affiché est encaissé en entier. Les fonds sont libérés après validation de la réception, c'est cette date-là qui compte au registre.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Défauts déclarés</t>
+          <t>Plus aucune ligne jaune</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
+          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
+          <t>Défauts déclarés</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
           <t>Import du Japon</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>La facture Meccha Japan #FA429713 ne porte aucune TVA. Si La Poste a réclamé la TVA à 20 % et des frais de dossier à la livraison, ce montant s'ajoute au coût d'achat : le noter en ligne séparée.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>OÙ VÉRIFIER</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>URSSAF</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Obligations du commerçant</t>
+          <t>URSSAF</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>entreprendre.service-public.fr</t>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>CGV et droit de la consommation</t>
+          <t>Obligations du commerçant</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+          <t>entreprendre.service-public.fr</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>
@@ -926,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K310"/>
+  <dimension ref="A1:K311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -974,7 +980,7 @@
         </is>
       </c>
       <c r="K4" s="6">
-        <f>SUM(E6:E310)</f>
+        <f>SUM(E6:E311)</f>
         <v/>
       </c>
     </row>
@@ -1217,28 +1223,32 @@
           <t>10/08/2026</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr"/>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Natalie Gulitz — Offenbach am Main, Allemagne</t>
+        </is>
+      </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>HAVAIANAS Slim — 2 paires à 14 €</t>
+          <t>HAVAIANAS Slim 35/36 — 1 paire</t>
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
-          <t>Espèces</t>
+          <t>Virement Vinted</t>
         </is>
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Main propre</t>
+          <t>Vinted</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Achat : FB2026-5844 lot n°120</t>
+          <t>Expédition Chronopost XU173687375JF du 03/08/2026 · achat FB2026-5844 lot n°120</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
@@ -1252,13 +1262,39 @@
         <f>IF(B11="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
-      <c r="H11" s="11" t="n"/>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>« Vintage Go » — pseudonyme Vinted</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>HAVAIANAS Slim 35/36 — 1 paire</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Virement Vinted</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Vinted</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Achat : FB2026-5844 lot n°120</t>
+        </is>
+      </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
           <t>À BASCULER dans le registre le jour du virement, pas avant.</t>
@@ -5254,8 +5290,21 @@
       <c r="G310" s="11" t="n"/>
       <c r="H310" s="11" t="n"/>
     </row>
+    <row r="311">
+      <c r="A311" s="10">
+        <f>IF(B311="","",ROW()-5)</f>
+        <v/>
+      </c>
+      <c r="B311" s="11" t="n"/>
+      <c r="C311" s="11" t="n"/>
+      <c r="D311" s="11" t="n"/>
+      <c r="E311" s="12" t="n"/>
+      <c r="F311" s="11" t="n"/>
+      <c r="G311" s="11" t="n"/>
+      <c r="H311" s="11" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:H310"/>
+  <autoFilter ref="A5:H311"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5486,7 +5535,7 @@
           <t>Lignes à compléter — fond jaune</t>
         </is>
       </c>
-      <c r="J8" s="15" t="n">
+      <c r="J8" s="14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -10578,7 +10627,7 @@
           <t>Objets inscrits</t>
         </is>
       </c>
-      <c r="N3" s="16">
+      <c r="N3" s="15">
         <f>COUNTIF(B6:B345,"&lt;&gt;")</f>
         <v/>
       </c>
@@ -10589,7 +10638,7 @@
           <t>Sortis du stock</t>
         </is>
       </c>
-      <c r="N4" s="16">
+      <c r="N4" s="15">
         <f>COUNT(J6:J345)</f>
         <v/>
       </c>
@@ -10808,104 +10857,104 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17">
+      <c r="A9" s="16">
         <f>IF(B9="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>ADN Enchères — Lyon</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Facture — opérateur de ventes volontaires agréé</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Lot de 12 paires de tongs HAVAIANAS fuchsia 35/36 — neuf</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Havaianas</t>
         </is>
       </c>
-      <c r="G9" s="19" t="n">
+      <c r="G9" s="18" t="n">
         <v>100.8</v>
       </c>
-      <c r="H9" s="18" t="inlineStr">
+      <c r="H9" s="17" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>10/08/2026</t>
         </is>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="J9" s="18" t="n">
         <v>28</v>
       </c>
-      <c r="K9" s="18" t="inlineStr">
-        <is>
-          <t>Sortie partielle : 2 paires sur 12, à 14 € l'unité</t>
+      <c r="K9" s="17" t="inlineStr">
+        <is>
+          <t>Sortie partielle : 2 paires sur 12 vendues sur Vinted à 14 € — 10 restent en stock</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17">
+      <c r="A10" s="16">
         <f>IF(B10="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="C10" s="18" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>ADN Enchères — Le Mans</t>
         </is>
       </c>
-      <c r="D10" s="18" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>Facture — opérateur de ventes volontaires agréé</t>
         </is>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>Veste en jean ARMANI EXCHANGE T.S — neuve</t>
         </is>
       </c>
-      <c r="F10" s="18" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Armani Exchange</t>
         </is>
       </c>
-      <c r="G10" s="19" t="n">
+      <c r="G10" s="18" t="n">
         <v>25.2</v>
       </c>
-      <c r="H10" s="18" t="inlineStr">
+      <c r="H10" s="17" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="I10" s="18" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>09/08/2026</t>
         </is>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="J10" s="18" t="n">
         <v>40</v>
       </c>
-      <c r="K10" s="18" t="inlineStr">
+      <c r="K10" s="17" t="inlineStr">
         <is>
           <t>Vendu à Mme Aouimeur Siham</t>
         </is>
@@ -11306,52 +11355,52 @@
       <c r="K19" s="11" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="17">
+      <c r="A20" s="16">
         <f>IF(B20="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>28/07/2026</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>ADN Enchères — Le Mans</t>
         </is>
       </c>
-      <c r="D20" s="18" t="inlineStr">
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Facture — opérateur de ventes volontaires agréé</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Sac demi-lune nylon noir KARL LAGERFELD JEANS — neuf avec étiquette</t>
         </is>
       </c>
-      <c r="F20" s="18" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Karl Lagerfeld Jeans</t>
         </is>
       </c>
-      <c r="G20" s="19" t="n">
+      <c r="G20" s="18" t="n">
         <v>50.4</v>
       </c>
-      <c r="H20" s="18" t="inlineStr">
+      <c r="H20" s="17" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="I20" s="18" t="inlineStr">
+      <c r="I20" s="17" t="inlineStr">
         <is>
           <t>09/08/2026</t>
         </is>
       </c>
-      <c r="J20" s="19" t="n">
+      <c r="J20" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="K20" s="18" t="inlineStr">
+      <c r="K20" s="17" t="inlineStr">
         <is>
           <t>Vendu à Mme Aouimeur Siham</t>
         </is>
@@ -11484,52 +11533,52 @@
       <c r="K23" s="11" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="17">
+      <c r="A24" s="16">
         <f>IF(B24="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>ADN Enchères — Lyon</t>
         </is>
       </c>
-      <c r="D24" s="18" t="inlineStr">
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>Facture — opérateur de ventes volontaires agréé</t>
         </is>
       </c>
-      <c r="E24" s="18" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>LACOSTE sneakers P.42 — neuves</t>
         </is>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>Lacoste</t>
         </is>
       </c>
-      <c r="G24" s="19" t="n">
+      <c r="G24" s="18" t="n">
         <v>57.51</v>
       </c>
-      <c r="H24" s="18" t="inlineStr">
+      <c r="H24" s="17" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
+      <c r="I24" s="17" t="inlineStr">
         <is>
           <t>09/08/2026</t>
         </is>
       </c>
-      <c r="J24" s="19" t="n">
+      <c r="J24" s="18" t="n">
         <v>70</v>
       </c>
-      <c r="K24" s="18" t="inlineStr">
+      <c r="K24" s="17" t="inlineStr">
         <is>
           <t>Vendu à Mme Aouimeur Siham</t>
         </is>
@@ -11872,52 +11921,52 @@
       <c r="K32" s="11" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="17">
+      <c r="A33" s="16">
         <f>IF(B33="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B33" s="18" t="inlineStr">
+      <c r="B33" s="17" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="C33" s="18" t="inlineStr">
+      <c r="C33" s="17" t="inlineStr">
         <is>
           <t>ADN Enchères — Le Mans</t>
         </is>
       </c>
-      <c r="D33" s="18" t="inlineStr">
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>Facture — opérateur de ventes volontaires agréé</t>
         </is>
       </c>
-      <c r="E33" s="18" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
         <is>
           <t>SALOMON X Ultra 5 Mid GTX P.44 — neuves</t>
         </is>
       </c>
-      <c r="F33" s="18" t="inlineStr">
+      <c r="F33" s="17" t="inlineStr">
         <is>
           <t>Salomon</t>
         </is>
       </c>
-      <c r="G33" s="19" t="n">
+      <c r="G33" s="18" t="n">
         <v>76.68000000000001</v>
       </c>
-      <c r="H33" s="18" t="inlineStr">
+      <c r="H33" s="17" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="I33" s="18" t="inlineStr">
+      <c r="I33" s="17" t="inlineStr">
         <is>
           <t>12/08/2026</t>
         </is>
       </c>
-      <c r="J33" s="19" t="n">
+      <c r="J33" s="18" t="n">
         <v>100</v>
       </c>
-      <c r="K33" s="18" t="inlineStr">
+      <c r="K33" s="17" t="inlineStr">
         <is>
           <t>Vendu, encaissement Vinted en attente</t>
         </is>
@@ -12008,52 +12057,52 @@
       <c r="K35" s="11" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="17">
+      <c r="A36" s="16">
         <f>IF(B36="","",ROW()-5)</f>
         <v/>
       </c>
-      <c r="B36" s="18" t="inlineStr">
+      <c r="B36" s="17" t="inlineStr">
         <is>
           <t>03/08/2026</t>
         </is>
       </c>
-      <c r="C36" s="18" t="inlineStr">
+      <c r="C36" s="17" t="inlineStr">
         <is>
           <t>ADN Enchères — Le Mans</t>
         </is>
       </c>
-      <c r="D36" s="18" t="inlineStr">
+      <c r="D36" s="17" t="inlineStr">
         <is>
           <t>Facture — opérateur de ventes volontaires agréé</t>
         </is>
       </c>
-      <c r="E36" s="18" t="inlineStr">
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>T-shirt BALENCIAGA T.2 — neuf</t>
         </is>
       </c>
-      <c r="F36" s="18" t="inlineStr">
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>Balenciaga</t>
         </is>
       </c>
-      <c r="G36" s="19" t="n">
+      <c r="G36" s="18" t="n">
         <v>113.4</v>
       </c>
-      <c r="H36" s="18" t="inlineStr">
+      <c r="H36" s="17" t="inlineStr">
         <is>
           <t>Carte</t>
         </is>
       </c>
-      <c r="I36" s="18" t="inlineStr">
+      <c r="I36" s="17" t="inlineStr">
         <is>
           <t>09/08/2026</t>
         </is>
       </c>
-      <c r="J36" s="19" t="n">
+      <c r="J36" s="18" t="n">
         <v>135</v>
       </c>
-      <c r="K36" s="18" t="inlineStr">
+      <c r="K36" s="17" t="inlineStr">
         <is>
           <t>Vendu à Mme Aouimeur Siham</t>
         </is>

</xml_diff>

<commit_message>
registres: justificatifs Vinted et releve annuel DAC7
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B43"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -833,89 +833,125 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Plus aucune ligne jaune</t>
+          <t>Justifier une vente Vinted</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
+          <t>Vinted n'affiche AUCUN numéro de commande au vendeur. Le justificatif, c'est l'historique du porte-monnaie (Profil puis Solde) : date, montant, article. En faire une capture d'écran. Le numéro de suivi du colis et la conversation avec l'acheteur complètent la preuve.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Défauts déclarés</t>
+          <t>Relevé annuel DAC7</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
+          <t>Vinted déclare au fisc les vendeurs dépassant 30 ventes ou 2 000 € par an, et envoie un relevé annuel récapitulatif vers janvier. Le conserver et VÉRIFIER QU'IL CONCORDE avec le livre des recettes : un écart entre ce que la plateforme déclare et ce que tu déclares est le premier déclencheur de contrôle.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Import du Japon</t>
+          <t>Exporter régulièrement</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>La facture Meccha Japan #FA429713 ne porte aucune TVA. Si La Poste a réclamé la TVA à 20 % et des frais de dossier à la livraison, ce montant s'ajoute au coût d'achat : le noter en ligne séparée.</t>
+          <t>Les plateformes ne gardent pas l'historique cinq ans, contrairement à l'obligation de conservation. Exporter les justificatifs en PDF ou en capture, dans un dossier daté.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Plus aucune ligne jaune</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>OÙ VÉRIFIER</t>
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Défauts déclarés</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>URSSAF</t>
+          <t>Import du Japon</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>Obligations du commerçant</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>entreprendre.service-public.fr</t>
+          <t>La facture Meccha Japan #FA429713 ne porte aucune TVA. Si La Poste a réclamé la TVA à 20 % et des frais de dossier à la livraison, ce montant s'ajoute au coût d'achat : le noter en ligne séparée.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>CGV et droit de la consommation</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>OÙ VÉRIFIER</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t>URSSAF</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Obligations du commerçant</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>entreprendre.service-public.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>
@@ -1248,7 +1284,7 @@
       </c>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>Expédition Chronopost XU173687375JF du 03/08/2026 · achat FB2026-5844 lot n°120</t>
+          <t>Vinted — suivi Chronopost XU173687375JF, expédiée le 03/08/2026</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
facture 2026-001 pour Mme Aouimeur Siham, 315 EUR
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -632,326 +632,338 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Conservation</t>
+          <t>Numérotation des factures</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>5 ans minimum. Garder les factures des maisons de vente, elles justifient chaque ligne.</t>
+          <t>Une seule série, continue, sans trou : 2026-001, 2026-002, 2026-003. Un numéro sauté ou réutilisé fait présumer une facture dissimulée. La première facture émise porte le n° 2026-001, vente à Mme Aouimeur Siham du 09/08/2026.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Sortie partielle</t>
+          <t>Conservation</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Un lot vendu à l'unité se solde en plusieurs fois : le noter en observations jusqu'à épuisement.</t>
+          <t>5 ans minimum. Garder les factures des maisons de vente, elles justifient chaque ligne.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Prélèvement personnel</t>
+          <t>Sortie partielle</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Un article gardé pour soi sort du stock sans recette. Il ne s'inscrit pas au livre des recettes — il n'y a pas d'encaissement — mais il se note en sortie sur le registre des objets mobiliers, avec la mention « usage personnel ». Sans cette ligne, le stock ne tombe jamais juste.</t>
+          <t>Un lot vendu à l'unité se solde en plusieurs fois : le noter en observations jusqu'à épuisement.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Le remboursement du prélèvement</t>
+          <t>Prélèvement personnel</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Remettre l'argent sur le compte pro n'est pas obligatoire — il n'y a qu'une personne juridique. Mais c'est une bonne pratique : sans ça, le stock fond et la caisse ne suit pas. Verser le COÛT D'ACHAT, pas le prix de vente : l'entreprise récupère ce qu'elle a payé, ni plus ni moins.</t>
+          <t>Un article gardé pour soi sort du stock sans recette. Il ne s'inscrit pas au livre des recettes — il n'y a pas d'encaissement — mais il se note en sortie sur le registre des objets mobiliers, avec la mention « usage personnel ». Sans cette ligne, le stock ne tombe jamais juste.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Apport, pas recette</t>
+          <t>Le remboursement du prélèvement</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Le virement du compte personnel vers le compte professionnel est un APPORT. Aucun chiffre d'affaires, aucune URSSAF, rien à déclarer. Le libeller « apport personnel » : sur un relevé pro, une somme qui arrive sans libellé ressemble à un encaissement client introuvable au livre des recettes.</t>
+          <t>Remettre l'argent sur le compte pro n'est pas obligatoire — il n'y a qu'une personne juridique. Mais c'est une bonne pratique : sans ça, le stock fond et la caisse ne suit pas. Verser le COÛT D'ACHAT, pas le prix de vente : l'entreprise récupère ce qu'elle a payé, ni plus ni moins.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
+          <t>Apport, pas recette</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Le virement du compte personnel vers le compte professionnel est un APPORT. Aucun chiffre d'affaires, aucune URSSAF, rien à déclarer. Le libeller « apport personnel » : sur un relevé pro, une somme qui arrive sans libellé ressemble à un encaissement client introuvable au livre des recettes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>Apport enregistré</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>150,50 € versés en apport personnel, couvrant au coût les quatre prélèvements : Hoka 65,37 € + Nike 52,77 € + pompe Robby ligne 131 19,41 € + booster High Class 12,95 €.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>VENTES EN ESPÈCES</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Plafond</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>1 000 € par transaction entre un professionnel et un particulier résidant en France — art. L112-6 du code monétaire et financier. Aucune vente n'en approche.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>La preuve</t>
+          <t>Plafond</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Une note de vente par transaction : date, article, prix, nom de l'acheteur. Un carnet à souches suffit. C'est elle qui adosse la ligne du registre.</t>
+          <t>1 000 € par transaction entre un professionnel et un particulier résidant en France — art. L112-6 du code monétaire et financier. Aucune vente n'en approche.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
+          <t>La preuve</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Une note de vente par transaction : date, article, prix, nom de l'acheteur. Un carnet à souches suffit. C'est elle qui adosse la ligne du registre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>Le dépôt</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Déposer directement sur le compte professionnel. Passer par le compte personnel puis virer casse le lien entre la vente et le relevé.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>DÉCLARATION URSSAF</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Ce qu'on déclare</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Le chiffre d'affaires encaissé sur la période. Total en haut à droite du livre des recettes.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Taux</t>
+          <t>Ce qu'on déclare</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>12,3 % de cotisations + 0,1 % de CFP = 12,4 %. À vérifier sur autoentrepreneur.urssaf.fr.</t>
+          <t>Le chiffre d'affaires encaissé sur la période. Total en haut à droite du livre des recettes.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Provision</t>
+          <t>Taux</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>À virer sur un compte séparé à chaque encaissement, pas au trimestre.</t>
+          <t>12,3 % de cotisations + 0,1 % de CFP = 12,4 %. À vérifier sur autoentrepreneur.urssaf.fr.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
+          <t>Provision</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>À virer sur un compte séparé à chaque encaissement, pas au trimestre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>Pas de versement libératoire</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>L'impôt suit le barème après abattement de 71 %. Il tombe l'année suivante — à provisionner aussi.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>CE QUI RESTE À COMPLÉTER</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Livre des recettes</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Complet. Quatre ventes à Mme Aouimeur Siham le 09/08 en espèces et main propre, deux paires de Havaianas sur Vinted encaissées le 10/08.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Ventes Vinted</t>
+          <t>Livre des recettes</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Sur un compte particulier, le vendeur ne paie pas de commission et l'acheteur paie le port : le prix affiché est encaissé en entier. Les fonds sont libérés après validation de la réception, c'est cette date-là qui compte au registre.</t>
+          <t>Complet. Quatre ventes à Mme Aouimeur Siham le 09/08 en espèces et main propre, deux paires de Havaianas sur Vinted encaissées le 10/08.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Justifier une vente Vinted</t>
+          <t>Ventes Vinted</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Vinted n'affiche AUCUN numéro de commande au vendeur. Le justificatif, c'est l'historique du porte-monnaie (Profil puis Solde) : date, montant, article. En faire une capture d'écran. Le numéro de suivi du colis et la conversation avec l'acheteur complètent la preuve.</t>
+          <t>Sur un compte particulier, le vendeur ne paie pas de commission et l'acheteur paie le port : le prix affiché est encaissé en entier. Les fonds sont libérés après validation de la réception, c'est cette date-là qui compte au registre.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Relevé annuel DAC7</t>
+          <t>Justifier une vente Vinted</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Vinted déclare au fisc les vendeurs dépassant 30 ventes ou 2 000 € par an, et envoie un relevé annuel récapitulatif vers janvier. Le conserver et VÉRIFIER QU'IL CONCORDE avec le livre des recettes : un écart entre ce que la plateforme déclare et ce que tu déclares est le premier déclencheur de contrôle.</t>
+          <t>Vinted n'affiche AUCUN numéro de commande au vendeur. Le justificatif, c'est l'historique du porte-monnaie (Profil puis Solde) : date, montant, article. En faire une capture d'écran. Le numéro de suivi du colis et la conversation avec l'acheteur complètent la preuve.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Exporter régulièrement</t>
+          <t>Relevé annuel DAC7</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Les plateformes ne gardent pas l'historique cinq ans, contrairement à l'obligation de conservation. Exporter les justificatifs en PDF ou en capture, dans un dossier daté.</t>
+          <t>Vinted déclare au fisc les vendeurs dépassant 30 ventes ou 2 000 € par an, et envoie un relevé annuel récapitulatif vers janvier. Le conserver et VÉRIFIER QU'IL CONCORDE avec le livre des recettes : un écart entre ce que la plateforme déclare et ce que tu déclares est le premier déclencheur de contrôle.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Plus aucune ligne jaune</t>
+          <t>Exporter régulièrement</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
+          <t>Les plateformes ne gardent pas l'historique cinq ans, contrairement à l'obligation de conservation. Exporter les justificatifs en PDF ou en capture, dans un dossier daté.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Défauts déclarés</t>
+          <t>Plus aucune ligne jaune</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
+          <t>Tous les achats ont leur facture. Bordereau ERA n°507148 réglé en deux fois : 59,60 € le 28/07 et 24,00 € le 03/08/2026.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
+          <t>Défauts déclarés</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>Deux pompes Robby portent un défaut mentionné au bordereau : socle cassé sur la ligne 122, mode manuel hors service sur la ligne 131. Le défaut se recopie dans l'annonce — un défaut caché se retourne contre le vendeur professionnel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
           <t>Import du Japon</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>La facture Meccha Japan #FA429713 ne porte aucune TVA. Si La Poste a réclamé la TVA à 20 % et des frais de dossier à la livraison, ce montant s'ajoute au coût d'achat : le noter en ligne séparée.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>OÙ VÉRIFIER</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>URSSAF</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Obligations du commerçant</t>
+          <t>URSSAF</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>entreprendre.service-public.fr</t>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>CGV et droit de la consommation</t>
+          <t>Obligations du commerçant</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+          <t>entreprendre.service-public.fr</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>
@@ -1106,7 +1118,7 @@
       </c>
       <c r="H6" s="11" t="inlineStr">
         <is>
-          <t>Achat : FB2026-44194 lot n°9</t>
+          <t>Facture n° 2026-001</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
@@ -1154,7 +1166,7 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>Achat : FB2026-43716 lot n°431</t>
+          <t>Facture n° 2026-001</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1205,7 @@
       </c>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>Achat : FB2026-6023 lot n°141</t>
+          <t>Facture n° 2026-001</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1237,7 +1249,7 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>Achat : FB2026-43717 lot n°168</t>
+          <t>Facture n° 2026-001</t>
         </is>
       </c>
       <c r="J9" s="8" t="inlineStr">

</xml_diff>

<commit_message>
facture 2026-001: SIRET et adresse client renseignes
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -917,53 +917,120 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>OÙ VÉRIFIER</t>
+          <t>IDENTITÉ DE L'ENTREPRISE</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>URSSAF</t>
+          <t>Exploitant</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
+          <t>Nacim IZRI — entrepreneur individuel (EI), enseigne Maison Nsaia.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>Obligations du commerçant</t>
+          <t>SIRET</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>entreprendre.service-public.fr</t>
+          <t>804 431 799 00027 — SIREN 804 431 799. Clé de contrôle vérifiée.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>CGV et droit de la consommation</t>
+          <t>RCS</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+          <t>RCS Toulouse 804 431 799. À confirmer sur l'extrait K : le greffe et le numéro doivent figurer sur toute facture d'un commerçant.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
+          <t>Siège</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>2 rue du Levant, 31700 Beauzelle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Mentions obligatoires sur facture</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Nom, mention « EI », adresse, SIRET, RCS, numéro et date de facture, identité du client, désignation et quantité, prix unitaire, total, « TVA non applicable, art. 293 B du CGI », date et mode de règlement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>OÙ VÉRIFIER</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>URSSAF</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Obligations du commerçant</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>entreprendre.service-public.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>

</xml_diff>

<commit_message>
facture: Maison Nsaia en identite, nom legal en mention discrete
</commit_message>
<xml_diff>
--- a/exports/maison-nsaia-registres.xlsx
+++ b/exports/maison-nsaia-registres.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B54"/>
+  <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -981,56 +981,80 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Enseigne et nom légal</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>« Maison Nsaia » est une ENSEIGNE, pas une société : elle s'ajoute au nom, elle ne le remplace jamais. L'entrepreneur individuel n'a pas de personnalité morale distincte — le vendeur, c'est la personne. Depuis mai 2022 (art. R526-27 du code de commerce), le nom doit figurer sur tous les documents commerciaux, suivi de « EI » ou « entrepreneur individuel ».</t>
+        </is>
+      </c>
+    </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>La mise en page permise</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>L'enseigne peut occuper l'en-tête et servir d'identité visuelle ; le nom légal descend en mention légale, en petits caractères. C'est ce que fait la facture 2026-001. Ce qui est interdit, c'est de le retirer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>OÙ VÉRIFIER</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="3" t="inlineStr">
-        <is>
-          <t>URSSAF</t>
-        </is>
-      </c>
-      <c r="B51" s="4" t="inlineStr">
-        <is>
-          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="3" t="inlineStr">
-        <is>
-          <t>Obligations du commerçant</t>
-        </is>
-      </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>entreprendre.service-public.fr</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>CGV et droit de la consommation</t>
+          <t>URSSAF</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+          <t>autoentrepreneur.urssaf.fr · téléphone 3698</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
+          <t>Obligations du commerçant</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>entreprendre.service-public.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>CGV et droit de la consommation</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>DGCCRF — economie.gouv.fr/dgccrf</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
           <t>Conseil gratuit</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
         <is>
           <t>Chambre de Commerce et d'Industrie — les conseillers reçoivent les commerçants sans frais.</t>
         </is>

</xml_diff>